<commit_message>
LLM response added - UI development next
</commit_message>
<xml_diff>
--- a/parser/data/xlsx/column_inspection.xlsx
+++ b/parser/data/xlsx/column_inspection.xlsx
@@ -5012,35 +5012,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>total_eve_charge</t>
+          <t>voice_mail_plan</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>total_day_charge</t>
+          <t>total_intl_charge</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>total_intl_charge</t>
+          <t>total_eve_charge</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>total_night_charge</t>
+          <t>total_day_charge</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>voice_mail_plan</t>
+          <t>total_night_charge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor changes in Backend
</commit_message>
<xml_diff>
--- a/parser/data/xlsx/column_inspection.xlsx
+++ b/parser/data/xlsx/column_inspection.xlsx
@@ -5012,35 +5012,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>voice_mail_plan</t>
+          <t>total_night_charge</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>total_intl_charge</t>
+          <t>total_eve_charge</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>total_eve_charge</t>
+          <t>total_day_charge</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>total_day_charge</t>
+          <t>voice_mail_plan</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>total_night_charge</t>
+          <t>total_intl_charge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor test pre-starting UI/UX
</commit_message>
<xml_diff>
--- a/parser/data/xlsx/column_inspection.xlsx
+++ b/parser/data/xlsx/column_inspection.xlsx
@@ -5012,35 +5012,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>total_night_charge</t>
+          <t>voice_mail_plan</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>total_eve_charge</t>
+          <t>total_intl_charge</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>total_day_charge</t>
+          <t>total_night_charge</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>voice_mail_plan</t>
+          <t>total_day_charge</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>total_intl_charge</t>
+          <t>total_eve_charge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI/UX Done - Final cleaning and testing remaining
</commit_message>
<xml_diff>
--- a/parser/data/xlsx/column_inspection.xlsx
+++ b/parser/data/xlsx/column_inspection.xlsx
@@ -434,7 +434,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>7abc486a8f2944fab510c38389cbf6f4.csv</t>
+          <t>5a6b5300428640cbaae38090de224504.csv</t>
         </is>
       </c>
     </row>
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C:\Users\Utkarsh Mishra\Downloads\Main Projects\Agentic_Auto_ML\uploaded_files\user_uploads\7abc486a8f2944fab510c38389cbf6f4.csv</t>
+          <t>C:\Users\Utkarsh Mishra\Downloads\Main Projects\Agentic_Auto_ML\uploaded_files\user_uploads\5a6b5300428640cbaae38090de224504.csv</t>
         </is>
       </c>
     </row>

</xml_diff>